<commit_message>
Changes made on 27 AUG
</commit_message>
<xml_diff>
--- a/SecureWipedocs/SecureWipe_Evidence_Tracker.xlsx
+++ b/SecureWipedocs/SecureWipe_Evidence_Tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parth goel\Downloads\SecureWipe_Project_Docs\SecureWipe\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parth goel\Desktop\SecureWipe\SecureWipedocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88305FC7-42D8-411F-AE60-51D6EFE19C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{105E7983-87B4-452D-9690-18AE0367340A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="81">
   <si>
     <t>ID</t>
   </si>
@@ -217,15 +217,9 @@
     <t>Partial</t>
   </si>
   <si>
-    <t>~35% per dev's own estimate</t>
-  </si>
-  <si>
     <t>F-17</t>
   </si>
   <si>
-    <t>Capability detection / Safety Engine / Policy Engine / Sanitization / Verification / Certificates</t>
-  </si>
-  <si>
     <t>PLANNED</t>
   </si>
   <si>
@@ -254,13 +248,34 @@
   </si>
   <si>
     <t xml:space="preserve">Vishal </t>
+  </si>
+  <si>
+    <t>Bus/device/media-type logic now exists, uses seek-penalty heuristic, not fully reliable yet</t>
+  </si>
+  <si>
+    <t>Capability Detection / Sanitization / Verification / Certificates</t>
+  </si>
+  <si>
+    <t>F-18</t>
+  </si>
+  <si>
+    <t>F-19</t>
+  </si>
+  <si>
+    <t>Safety Engine foundation</t>
+  </si>
+  <si>
+    <t>Qt Desktop</t>
+  </si>
+  <si>
+    <t>System-disk + physical-device checks partially working, boot/mounted-volume/OS-dependency not implemented</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -284,6 +299,12 @@
       <b/>
       <sz val="13"/>
       <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -587,7 +608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -877,7 +898,7 @@
         <v>13</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>15</v>
@@ -906,7 +927,7 @@
         <v>13</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>15</v>
@@ -1063,7 +1084,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>60</v>
       </c>
@@ -1089,24 +1110,24 @@
       </c>
       <c r="J17" s="2"/>
       <c r="K17" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="B18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="D18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>67</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -1114,14 +1135,53 @@
         <v>25</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2" t="s">
-        <v>68</v>
-      </c>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="57" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K20" s="2"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="C2:C500" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"DONE,TESTED,IN PROGRESS,PLANNED"</formula1>
@@ -1143,7 +1203,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -1151,22 +1211,22 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes made till 28AUG
</commit_message>
<xml_diff>
--- a/SecureWipedocs/SecureWipe_Evidence_Tracker.xlsx
+++ b/SecureWipedocs/SecureWipe_Evidence_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parth goel\Desktop\SecureWipe\SecureWipedocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{105E7983-87B4-452D-9690-18AE0367340A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCE76729-33AD-4382-8C5F-A5CA09EC8E0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="112">
   <si>
     <t>ID</t>
   </si>
@@ -269,6 +269,99 @@
   </si>
   <si>
     <t>System-disk + physical-device checks partially working, boot/mounted-volume/OS-dependency not implemented</t>
+  </si>
+  <si>
+    <t>F-20</t>
+  </si>
+  <si>
+    <t>F-21</t>
+  </si>
+  <si>
+    <t>Workstation ↔ Workstation Center linking</t>
+  </si>
+  <si>
+    <t>Sanitization request (create/view, PENDING status)</t>
+  </si>
+  <si>
+    <t>Approval/assignment/wipe/verify/cert not built</t>
+  </si>
+  <si>
+    <t>F-22</t>
+  </si>
+  <si>
+    <t>Desktop Device Details page</t>
+  </si>
+  <si>
+    <t>Capacity shows 0 B (backend bug), no SafetyEngine integration yet</t>
+  </si>
+  <si>
+    <t>F-23</t>
+  </si>
+  <si>
+    <t>F-24</t>
+  </si>
+  <si>
+    <t>F-25</t>
+  </si>
+  <si>
+    <t>F-26</t>
+  </si>
+  <si>
+    <t>BCD→physical disk mapping still missing — boot-disk protection not fully reliable yet</t>
+  </si>
+  <si>
+    <t>Folder created only, EvidenceItem not built</t>
+  </si>
+  <si>
+    <t>WindowsStorageUtils layer</t>
+  </si>
+  <si>
+    <t>Target Identity / SafetyEngine core validation</t>
+  </si>
+  <si>
+    <t>Windows BCD/system-partition detection</t>
+  </si>
+  <si>
+    <t>Evidence structure</t>
+  </si>
+  <si>
+    <t>F-27</t>
+  </si>
+  <si>
+    <t>F-28</t>
+  </si>
+  <si>
+    <t>Structured SafetyResult reporting</t>
+  </si>
+  <si>
+    <t>Boot Dependency check (WindowsBootChecker)</t>
+  </si>
+  <si>
+    <t>Designed, not fully integration-tested</t>
+  </si>
+  <si>
+    <t>Sanitization will require overall SAFE result once finished</t>
+  </si>
+  <si>
+    <t>Same gap as 27 Aug — BCD→physical-disk mapping unresolved</t>
+  </si>
+  <si>
+    <t>F-29</t>
+  </si>
+  <si>
+    <t>F-30</t>
+  </si>
+  <si>
+    <t>Request approval/rejection workflow</t>
+  </si>
+  <si>
+    <t>Employee + Workstation assignment workflow</t>
+  </si>
+  <si>
+    <t>Returns HTTP 200</t>
+  </si>
+  <si>
+    <t>Validates role/active/center-ownership/availability</t>
   </si>
 </sst>
 </file>
@@ -608,7 +701,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1179,6 +1272,217 @@
         <v>15</v>
       </c>
       <c r="K20" s="2"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="42.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B23" t="s">
+        <v>87</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B25" t="s">
+        <v>96</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K25" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B27" t="s">
+        <v>98</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="K27" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="K28" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B29" t="s">
+        <v>102</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K29" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K30" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B31" t="s">
+        <v>109</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K31" t="s">
+        <v>111</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>

<commit_message>
resolve merge conflicts in sanitization backend
</commit_message>
<xml_diff>
--- a/SecureWipedocs/SecureWipe_Evidence_Tracker.xlsx
+++ b/SecureWipedocs/SecureWipe_Evidence_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parth goel\Desktop\SecureWipe\SecureWipedocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{105E7983-87B4-452D-9690-18AE0367340A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCE76729-33AD-4382-8C5F-A5CA09EC8E0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="112">
   <si>
     <t>ID</t>
   </si>
@@ -269,6 +269,99 @@
   </si>
   <si>
     <t>System-disk + physical-device checks partially working, boot/mounted-volume/OS-dependency not implemented</t>
+  </si>
+  <si>
+    <t>F-20</t>
+  </si>
+  <si>
+    <t>F-21</t>
+  </si>
+  <si>
+    <t>Workstation ↔ Workstation Center linking</t>
+  </si>
+  <si>
+    <t>Sanitization request (create/view, PENDING status)</t>
+  </si>
+  <si>
+    <t>Approval/assignment/wipe/verify/cert not built</t>
+  </si>
+  <si>
+    <t>F-22</t>
+  </si>
+  <si>
+    <t>Desktop Device Details page</t>
+  </si>
+  <si>
+    <t>Capacity shows 0 B (backend bug), no SafetyEngine integration yet</t>
+  </si>
+  <si>
+    <t>F-23</t>
+  </si>
+  <si>
+    <t>F-24</t>
+  </si>
+  <si>
+    <t>F-25</t>
+  </si>
+  <si>
+    <t>F-26</t>
+  </si>
+  <si>
+    <t>BCD→physical disk mapping still missing — boot-disk protection not fully reliable yet</t>
+  </si>
+  <si>
+    <t>Folder created only, EvidenceItem not built</t>
+  </si>
+  <si>
+    <t>WindowsStorageUtils layer</t>
+  </si>
+  <si>
+    <t>Target Identity / SafetyEngine core validation</t>
+  </si>
+  <si>
+    <t>Windows BCD/system-partition detection</t>
+  </si>
+  <si>
+    <t>Evidence structure</t>
+  </si>
+  <si>
+    <t>F-27</t>
+  </si>
+  <si>
+    <t>F-28</t>
+  </si>
+  <si>
+    <t>Structured SafetyResult reporting</t>
+  </si>
+  <si>
+    <t>Boot Dependency check (WindowsBootChecker)</t>
+  </si>
+  <si>
+    <t>Designed, not fully integration-tested</t>
+  </si>
+  <si>
+    <t>Sanitization will require overall SAFE result once finished</t>
+  </si>
+  <si>
+    <t>Same gap as 27 Aug — BCD→physical-disk mapping unresolved</t>
+  </si>
+  <si>
+    <t>F-29</t>
+  </si>
+  <si>
+    <t>F-30</t>
+  </si>
+  <si>
+    <t>Request approval/rejection workflow</t>
+  </si>
+  <si>
+    <t>Employee + Workstation assignment workflow</t>
+  </si>
+  <si>
+    <t>Returns HTTP 200</t>
+  </si>
+  <si>
+    <t>Validates role/active/center-ownership/availability</t>
   </si>
 </sst>
 </file>
@@ -608,7 +701,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1179,6 +1272,217 @@
         <v>15</v>
       </c>
       <c r="K20" s="2"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="42.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B23" t="s">
+        <v>87</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B25" t="s">
+        <v>96</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K25" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B27" t="s">
+        <v>98</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="K27" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="K28" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B29" t="s">
+        <v>102</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K29" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K30" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B31" t="s">
+        <v>109</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K31" t="s">
+        <v>111</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>

<commit_message>
Documentatio till 2nd sep
</commit_message>
<xml_diff>
--- a/SecureWipedocs/SecureWipe_Evidence_Tracker.xlsx
+++ b/SecureWipedocs/SecureWipe_Evidence_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parth goel\Desktop\SecureWipe\SecureWipedocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCE76729-33AD-4382-8C5F-A5CA09EC8E0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B174B83-3E96-4DB9-BC97-C5187178D08F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="146">
   <si>
     <t>ID</t>
   </si>
@@ -362,13 +362,115 @@
   </si>
   <si>
     <t>Validates role/active/center-ownership/availability</t>
+  </si>
+  <si>
+    <t>F-31</t>
+  </si>
+  <si>
+    <t>F-32</t>
+  </si>
+  <si>
+    <t>Sequential IDs (CTR-/WS-/REQ-) via Counter model</t>
+  </si>
+  <si>
+    <t>Workstation Head Dashboard (Centre ID + Requests section)</t>
+  </si>
+  <si>
+    <t>F-33</t>
+  </si>
+  <si>
+    <t>F-34</t>
+  </si>
+  <si>
+    <t>F-35</t>
+  </si>
+  <si>
+    <t>Eligible-employee lookup API</t>
+  </si>
+  <si>
+    <t>Employee assigned-requests API</t>
+  </si>
+  <si>
+    <t>Employee status transition API (ASSIGNED→...→COMPLETED/FAILED)</t>
+  </si>
+  <si>
+    <t>Enforces ownership + valid transitions only</t>
+  </si>
+  <si>
+    <t>Desktop employee auth + assigned-jobs dashboard</t>
+  </si>
+  <si>
+    <t>F-36</t>
+  </si>
+  <si>
+    <t>Confirmed 403 correctly blocks non-employee roles</t>
+  </si>
+  <si>
+    <t>Sanitization capability detection (SCSI/storage-property queries)</t>
+  </si>
+  <si>
+    <t>F-37</t>
+  </si>
+  <si>
+    <t>Both real devices tested; native-sanitize support came back UNKNOWN for both, not a failure</t>
+  </si>
+  <si>
+    <t>NVMe Sanitize command implementation</t>
+  </si>
+  <si>
+    <t>F-38</t>
+  </si>
+  <si>
+    <t>F-39</t>
+  </si>
+  <si>
+    <t>Sanitization ↔ Safety Engine integration</t>
+  </si>
+  <si>
+    <t>Compiles, not run on real hardware yet</t>
+  </si>
+  <si>
+    <t>Do not claim sanitization works yet</t>
+  </si>
+  <si>
+    <t>Sanitize now blocked unless safety checks pass</t>
+  </si>
+  <si>
+    <t>F-40</t>
+  </si>
+  <si>
+    <t>F-41</t>
+  </si>
+  <si>
+    <t>Chunk-based JPEG carving (EvidenceCollector)</t>
+  </si>
+  <si>
+    <t>EvidenceItem data model</t>
+  </si>
+  <si>
+    <t>Recovered real JPEGs from a 62GB USB drive, including one across a chunk boundary</t>
+  </si>
+  <si>
+    <t>Not tested -data structure only</t>
+  </si>
+  <si>
+    <t>No carving/validation/scoring logic yet</t>
+  </si>
+  <si>
+    <t>F-42</t>
+  </si>
+  <si>
+    <t>Desktop request selection → Wipe page wiring</t>
+  </si>
+  <si>
+    <t>UI checkpoint only, no actual sanitization triggered yet</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -400,6 +502,17 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -427,7 +540,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -437,6 +550,13 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -701,7 +821,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1482,6 +1602,231 @@
       </c>
       <c r="K31" t="s">
         <v>111</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B33" t="s">
+        <v>115</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B35" t="s">
+        <v>120</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="42.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K36" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B37" t="s">
+        <v>123</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K37" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K38" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="42.75" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B39" t="s">
+        <v>129</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K39" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K40" s="5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B41" t="s">
+        <v>138</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="K41" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="K42" s="5" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B43" t="s">
+        <v>144</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="K43" t="s">
+        <v>145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>